<commit_message>
kea and tui integrated in parscen
</commit_message>
<xml_diff>
--- a/ReportDefs_vervestacks.xlsx
+++ b/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_NZL_EECA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A5049DA-4A1C-4846-AA89-387D28D5F3B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027CE7CB-80BD-4CCE-BF53-D2903CD42A24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="4" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3271" uniqueCount="1212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3272" uniqueCount="1213">
   <si>
     <t>Unit</t>
   </si>
@@ -3720,6 +3720,9 @@
   </si>
   <si>
     <t>Green Hydrogen Fuel</t>
+  </si>
+  <si>
+    <t>-ev_bat*</t>
   </si>
 </sst>
 </file>
@@ -21349,6 +21352,9 @@
       <c r="A23" t="s">
         <v>160</v>
       </c>
+      <c r="D23" s="2" t="s">
+        <v>1212</v>
+      </c>
       <c r="H23" t="s">
         <v>1015</v>
       </c>

</xml_diff>